<commit_message>
Update rdk8 components page
Signed-off-by: Dhanapal Raju <ldhana149@cable.comcast.com>
</commit_message>
<xml_diff>
--- a/video/rdk8/RDK8-comonents-catalog-draft.xlsx
+++ b/video/rdk8/RDK8-comonents-catalog-draft.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ldhana149\rdk-core-specs\video\rdk8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D432A5E2-C178-4CB0-970B-1DEB36F39ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD896CB-5E2C-456B-BCCA-019BF049BEB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{25E4EBF0-253B-4C9C-998E-FB08C73FD49A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$58</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="237">
   <si>
     <t>COMPONENTS</t>
   </si>
@@ -723,6 +723,36 @@
   </si>
   <si>
     <t>https://github.com/rdkcentral/Ripple</t>
+  </si>
+  <si>
+    <t>Breakpad Wrapper</t>
+  </si>
+  <si>
+    <t>https://code.rdkcentral.com/r/plugins/gitiles/rdk/components/generic/breakpad_wrapper</t>
+  </si>
+  <si>
+    <t>6.0.1</t>
+  </si>
+  <si>
+    <t>HDMI CEC Header</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-halif-hdmi_cec</t>
+  </si>
+  <si>
+    <t>Lisa</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/LISA</t>
+  </si>
+  <si>
+    <t>RDK GStreamer Utils</t>
+  </si>
+  <si>
+    <t>Video</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-gstreamer-utils-raspberrypi</t>
   </si>
 </sst>
 </file>
@@ -890,7 +920,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="21">
     <dxf>
       <font>
         <color theme="1"/>
@@ -953,6 +983,136 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1286,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8248C6F-D34E-4152-91E6-D60E20A6E179}">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1438,288 +1598,288 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B11" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="8" t="s">
+      <c r="C11" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="5" t="s">
+      <c r="C12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B13" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="8" t="s">
+      <c r="C13" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="5" t="s">
+      <c r="C14" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>122</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B16" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="8" t="s">
+      <c r="C16" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F16" s="8" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="5" t="s">
+      <c r="C17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B19" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="8" t="s">
+      <c r="C19" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F19" s="8" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E19" s="5" t="s">
+      <c r="C20" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>21</v>
+        <v>229</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>19</v>
@@ -1731,15 +1891,15 @@
         <v>7</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>19</v>
@@ -1751,55 +1911,55 @@
         <v>7</v>
       </c>
       <c r="E23" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F24" s="10" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B25" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E24" s="5" t="s">
+      <c r="C25" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>147</v>
@@ -1811,118 +1971,118 @@
         <v>7</v>
       </c>
       <c r="E26" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F27" s="10" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="5" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B28" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="5" t="s">
+      <c r="C28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F28" s="7" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="8" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B29" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" s="8" t="s">
+      <c r="C29" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F29" s="10" t="s">
         <v>153</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>155</v>
+        <v>82</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>116</v>
+        <v>19</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="5">
-        <v>2.35</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>156</v>
+      <c r="E30" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>158</v>
+        <v>116</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E31" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>159</v>
+      <c r="E31" s="5">
+        <v>2.35</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>6</v>
@@ -1933,36 +2093,36 @@
       <c r="E32" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>162</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>105</v>
+        <v>161</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>6</v>
@@ -1971,18 +2131,18 @@
         <v>7</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F34" s="10" t="s">
-        <v>164</v>
+        <v>59</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>19</v>
+        <v>105</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>6</v>
@@ -1991,15 +2151,15 @@
         <v>7</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>165</v>
+        <v>33</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>166</v>
+        <v>84</v>
       </c>
       <c r="B36" s="8" t="s">
         <v>19</v>
@@ -2011,18 +2171,18 @@
         <v>7</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>168</v>
+        <v>26</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>169</v>
+        <v>230</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>19</v>
+        <v>105</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>6</v>
@@ -2031,178 +2191,176 @@
         <v>7</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>170</v>
+        <v>30</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>116</v>
+        <v>19</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>173</v>
+        <v>167</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>43</v>
+        <v>169</v>
       </c>
       <c r="B39" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C39" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>174</v>
+      <c r="C40" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" s="9"/>
+      <c r="E41" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B44" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="C41" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E41" s="8" t="s">
+      <c r="C44" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F41" s="8" t="s">
+      <c r="F44" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="8" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B45" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C45" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="8" t="s">
+      <c r="D45" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E45" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="F42" s="8" t="s">
+      <c r="F45" s="8" t="s">
         <v>179</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F43" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>6</v>
@@ -2211,118 +2369,116 @@
         <v>7</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>184</v>
+        <v>73</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B50" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C50" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D47" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E47" s="5" t="s">
+      <c r="D50" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F50" s="5" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F48" s="8" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F50" s="8" t="s">
-        <v>188</v>
-      </c>
-    </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>189</v>
+      <c r="A51" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D51" s="6"/>
+      <c r="E51" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>175</v>
+        <v>130</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>6</v>
@@ -2331,58 +2487,58 @@
         <v>7</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>190</v>
+        <v>52</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>191</v>
+        <v>88</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>38</v>
+        <v>116</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>7</v>
       </c>
       <c r="E53" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A54" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E54" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F53" s="7" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>195</v>
+      <c r="F54" s="8" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="8" t="s">
-        <v>196</v>
+        <v>54</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>6</v>
@@ -2391,18 +2547,18 @@
         <v>7</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F55" s="8" t="s">
-        <v>197</v>
+        <v>55</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>6</v>
@@ -2411,18 +2567,18 @@
         <v>7</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F56" s="8" t="s">
-        <v>198</v>
+        <v>56</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>35</v>
+        <v>191</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>161</v>
+        <v>38</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>6</v>
@@ -2431,18 +2587,18 @@
         <v>7</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>37</v>
+        <v>8</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>41</v>
+        <v>193</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>199</v>
+        <v>116</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>6</v>
@@ -2451,18 +2607,18 @@
         <v>7</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>40</v>
+        <v>194</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>147</v>
+        <v>112</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>6</v>
@@ -2471,58 +2627,58 @@
         <v>7</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="F59" s="11" t="s">
-        <v>226</v>
+        <v>57</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>203</v>
+      <c r="A60" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C61" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F61" s="8" t="s">
-        <v>205</v>
+      <c r="A61" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>206</v>
+        <v>41</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>6</v>
@@ -2531,18 +2687,18 @@
         <v>7</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>207</v>
+        <v>40</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="8" t="s">
-        <v>42</v>
+        <v>200</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>209</v>
+        <v>147</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>6</v>
@@ -2551,161 +2707,161 @@
         <v>7</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F63" s="8" t="s">
-        <v>210</v>
+        <v>201</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>65</v>
+        <v>202</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>147</v>
+        <v>19</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E64" s="5">
-        <v>230</v>
+      <c r="E64" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>212</v>
+      <c r="A65" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="B66" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C66" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D66" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E66" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F66" s="8" t="s">
-        <v>62</v>
+      <c r="A66" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="8" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>116</v>
+        <v>209</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>214</v>
+        <v>65</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D68" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E68" s="5" t="s">
+      <c r="E68" s="5">
+        <v>230</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E70" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F68" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B69" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C69" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="F69" s="8" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D70" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F70" s="7" t="s">
-        <v>218</v>
+      <c r="F70" s="8" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="8" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="B71" s="8" t="s">
         <v>116</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D71" s="9" t="s">
         <v>7</v>
@@ -2713,16 +2869,16 @@
       <c r="E71" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F71" s="10" t="s">
-        <v>63</v>
+      <c r="F71" s="8" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>6</v>
@@ -2731,147 +2887,277 @@
         <v>7</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F72" s="7" t="s">
-        <v>220</v>
+        <v>8</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B73" s="5" t="s">
+      <c r="A73" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C73" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E73" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>221</v>
+      <c r="C73" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F73" s="8" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F75" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F77" s="5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B78" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C74" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E74" s="5" t="s">
+      <c r="C78" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F78" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A75" s="5" t="s">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="B79" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C75" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D75" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E75" s="5" t="s">
+      <c r="C79" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E79" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F79" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A76" s="8" t="s">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B76" s="8" t="s">
+      <c r="B80" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C76" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D76" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E76" s="8" t="s">
+      <c r="C80" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E80" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F76" s="8" t="s">
+      <c r="F80" s="8" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A77" s="12" t="s">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B81" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C77" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E77" s="13" t="s">
+      <c r="C81" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E81" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F77" s="12" t="s">
+      <c r="F81" s="12" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A78" s="14" t="s">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="B78" s="14" t="s">
+      <c r="B82" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C78" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E78" s="15" t="s">
+      <c r="C82" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E82" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F78" s="14" t="s">
+      <c r="F82" s="14" t="s">
         <v>225</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A54" xr:uid="{D8248C6F-D34E-4152-91E6-D60E20A6E179}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F54">
-      <sortCondition ref="A1:A54"/>
+  <autoFilter ref="A1:A58" xr:uid="{D8248C6F-D34E-4152-91E6-D60E20A6E179}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F58">
+      <sortCondition ref="A1:A58"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="D2:E78">
+  <conditionalFormatting sqref="C2:D7 C9:D36 C38:D82">
+    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
+      <formula>"vendor"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="23" operator="equal">
+      <formula>"oss"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="24" operator="equal">
+      <formula>"application"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="25" operator="equal">
+      <formula>"assembler"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="26" operator="equal">
+      <formula>"middleware"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E7 D9:E36 D38:E82">
+    <cfRule type="cellIs" dxfId="15" priority="27" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="28" operator="containsText" text="Y">
+      <formula>NOT(ISERROR(SEARCH("Y",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8:E8">
+    <cfRule type="cellIs" dxfId="13" priority="20" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="21" operator="containsText" text="Y">
+      <formula>NOT(ISERROR(SEARCH("Y",D8)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8:D8">
+    <cfRule type="cellIs" dxfId="11" priority="15" operator="equal">
+      <formula>"vendor"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="16" operator="equal">
+      <formula>"oss"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="17" operator="equal">
+      <formula>"application"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="18" operator="equal">
+      <formula>"assembler"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="19" operator="equal">
+      <formula>"middleware"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D37:E37">
     <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="Y">
-      <formula>NOT(ISERROR(SEARCH("Y",D2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Y",D37)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:D78">
+  <conditionalFormatting sqref="C37:D37">
     <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"vendor"</formula>
     </cfRule>
@@ -2889,7 +3175,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:D78" xr:uid="{99954803-2B18-46A2-978C-692392E0C4B3}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:D82" xr:uid="{99954803-2B18-46A2-978C-692392E0C4B3}">
       <formula1>"application, middleware, vendor, oss, assembler,config/manifest"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2899,30 +3185,33 @@
     <hyperlink ref="F5" r:id="rId3" xr:uid="{C1C242CB-5D2F-4955-9927-ED01C63BBF77}"/>
     <hyperlink ref="F6" r:id="rId4" xr:uid="{01985D25-D3D0-414C-9C6D-F6658A51F2C8}"/>
     <hyperlink ref="F4" r:id="rId5" xr:uid="{1EB2E145-C8FC-4797-A406-D266988A5E32}"/>
-    <hyperlink ref="F9" r:id="rId6" xr:uid="{7093F051-070F-480C-B763-0D2054B2629E}"/>
-    <hyperlink ref="F16" r:id="rId7" xr:uid="{6B3C3493-D21E-42A7-B8F5-F03C2413BF8D}"/>
-    <hyperlink ref="F24" r:id="rId8" xr:uid="{C9352B2C-55D0-4C58-8433-C23DE4753386}"/>
-    <hyperlink ref="F20" r:id="rId9" xr:uid="{3B14BD40-537E-43C8-99AB-8C196221B517}"/>
-    <hyperlink ref="F23" r:id="rId10" xr:uid="{4780326E-EE92-4F0F-B9D3-55DEA9DCFB8E}"/>
-    <hyperlink ref="F22" r:id="rId11" xr:uid="{D055BFCB-4982-45B6-A120-912BD5848209}"/>
-    <hyperlink ref="F21" r:id="rId12" xr:uid="{75CB34CD-61B8-49DB-8921-C0F71BE4D21E}"/>
-    <hyperlink ref="F26" r:id="rId13" xr:uid="{2F3895E8-1106-43EB-BD0A-3A6124FD442D}"/>
-    <hyperlink ref="F28" r:id="rId14" xr:uid="{19A4D98C-E8FE-4802-82C0-1784E93E130F}"/>
-    <hyperlink ref="F29" r:id="rId15" xr:uid="{01EF30D9-90B1-4432-B6E1-FA2D06886E34}"/>
-    <hyperlink ref="F27" r:id="rId16" xr:uid="{3D9F4E57-CD33-42F0-AAD5-C90018B3EE70}"/>
-    <hyperlink ref="F31" r:id="rId17" xr:uid="{B0ABB7E1-748F-4AC8-AF82-51956AC51067}"/>
-    <hyperlink ref="F34" r:id="rId18" xr:uid="{5D3B7B52-5FF8-4870-8BAF-B5CA79534C11}"/>
-    <hyperlink ref="F36" r:id="rId19" xr:uid="{99082EFD-1C79-4737-868C-4635BC596A4B}"/>
-    <hyperlink ref="F37" r:id="rId20" xr:uid="{7E547506-4CEE-4D92-A839-D0F2114F3850}"/>
-    <hyperlink ref="F39" r:id="rId21" xr:uid="{21021571-C052-41DD-A49F-A9703DC4A3FB}"/>
-    <hyperlink ref="F46" r:id="rId22" xr:uid="{AE6DE287-BAFE-4D20-942B-3AC2B766C643}"/>
-    <hyperlink ref="F59" r:id="rId23" xr:uid="{B8CB95C2-C6DB-4BAC-BAFC-7C71023397E0}"/>
-    <hyperlink ref="F51" r:id="rId24" xr:uid="{DAADDF7F-1222-4702-88B4-5BB31313EE66}"/>
-    <hyperlink ref="F53" r:id="rId25" xr:uid="{E2F05D0E-F1DA-4194-8A06-BB7FC0235DFF}"/>
-    <hyperlink ref="F52" r:id="rId26" xr:uid="{1B3DCB3D-6879-4C99-BFAC-74FCF8A81313}"/>
-    <hyperlink ref="F70" r:id="rId27" xr:uid="{5D056AD0-38A8-4E91-9AB8-5DDB725986C5}"/>
-    <hyperlink ref="F71" r:id="rId28" xr:uid="{B48BB988-25A9-4597-A9A3-DA7F75B413B8}"/>
-    <hyperlink ref="F72" r:id="rId29" xr:uid="{2B822696-CA69-4AA3-9BD8-95A76796E766}"/>
+    <hyperlink ref="F10" r:id="rId6" xr:uid="{7093F051-070F-480C-B763-0D2054B2629E}"/>
+    <hyperlink ref="F17" r:id="rId7" xr:uid="{6B3C3493-D21E-42A7-B8F5-F03C2413BF8D}"/>
+    <hyperlink ref="F25" r:id="rId8" xr:uid="{C9352B2C-55D0-4C58-8433-C23DE4753386}"/>
+    <hyperlink ref="F21" r:id="rId9" xr:uid="{3B14BD40-537E-43C8-99AB-8C196221B517}"/>
+    <hyperlink ref="F24" r:id="rId10" xr:uid="{4780326E-EE92-4F0F-B9D3-55DEA9DCFB8E}"/>
+    <hyperlink ref="F23" r:id="rId11" xr:uid="{D055BFCB-4982-45B6-A120-912BD5848209}"/>
+    <hyperlink ref="F22" r:id="rId12" xr:uid="{75CB34CD-61B8-49DB-8921-C0F71BE4D21E}"/>
+    <hyperlink ref="F27" r:id="rId13" xr:uid="{2F3895E8-1106-43EB-BD0A-3A6124FD442D}"/>
+    <hyperlink ref="F29" r:id="rId14" xr:uid="{19A4D98C-E8FE-4802-82C0-1784E93E130F}"/>
+    <hyperlink ref="F30" r:id="rId15" xr:uid="{01EF30D9-90B1-4432-B6E1-FA2D06886E34}"/>
+    <hyperlink ref="F28" r:id="rId16" xr:uid="{3D9F4E57-CD33-42F0-AAD5-C90018B3EE70}"/>
+    <hyperlink ref="F32" r:id="rId17" xr:uid="{B0ABB7E1-748F-4AC8-AF82-51956AC51067}"/>
+    <hyperlink ref="F35" r:id="rId18" xr:uid="{5D3B7B52-5FF8-4870-8BAF-B5CA79534C11}"/>
+    <hyperlink ref="F38" r:id="rId19" xr:uid="{99082EFD-1C79-4737-868C-4635BC596A4B}"/>
+    <hyperlink ref="F39" r:id="rId20" xr:uid="{7E547506-4CEE-4D92-A839-D0F2114F3850}"/>
+    <hyperlink ref="F42" r:id="rId21" xr:uid="{21021571-C052-41DD-A49F-A9703DC4A3FB}"/>
+    <hyperlink ref="F49" r:id="rId22" xr:uid="{AE6DE287-BAFE-4D20-942B-3AC2B766C643}"/>
+    <hyperlink ref="F63" r:id="rId23" xr:uid="{B8CB95C2-C6DB-4BAC-BAFC-7C71023397E0}"/>
+    <hyperlink ref="F55" r:id="rId24" xr:uid="{DAADDF7F-1222-4702-88B4-5BB31313EE66}"/>
+    <hyperlink ref="F57" r:id="rId25" xr:uid="{E2F05D0E-F1DA-4194-8A06-BB7FC0235DFF}"/>
+    <hyperlink ref="F56" r:id="rId26" xr:uid="{1B3DCB3D-6879-4C99-BFAC-74FCF8A81313}"/>
+    <hyperlink ref="F74" r:id="rId27" xr:uid="{5D056AD0-38A8-4E91-9AB8-5DDB725986C5}"/>
+    <hyperlink ref="F75" r:id="rId28" xr:uid="{B48BB988-25A9-4597-A9A3-DA7F75B413B8}"/>
+    <hyperlink ref="F76" r:id="rId29" xr:uid="{2B822696-CA69-4AA3-9BD8-95A76796E766}"/>
+    <hyperlink ref="F37" r:id="rId30" xr:uid="{A26FEA9E-3E64-4A90-A64E-E87CC96731C1}"/>
+    <hyperlink ref="F41" r:id="rId31" xr:uid="{3199F15F-D415-4AD0-A073-4EA06EFB8372}"/>
+    <hyperlink ref="F51" r:id="rId32" xr:uid="{4FB3C80E-6066-4425-A2F2-A87BD77D2B70}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>